<commit_message>
Update README and improve repository security
</commit_message>
<xml_diff>
--- a/reports.xlsx
+++ b/reports.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,383 +436,354 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1776587356615</v>
+        <v>1713510000000</v>
       </c>
       <c r="B2" t="str">
-        <v>19/4/2026</v>
+        <v>18/4/2026</v>
       </c>
       <c r="C2" t="str">
-        <v>Pending</v>
+        <v>Verified Fake</v>
       </c>
       <c r="D2" t="str">
-        <v>Baswaraj_Mundkar</v>
+        <v>Rahul_Sharma</v>
       </c>
       <c r="E2" t="str">
-        <v>Breaking news earthquake</v>
+        <v>WhatsApp forward claiming garlic cures the new virus</v>
       </c>
       <c r="F2" t="str">
-        <v>Instagram</v>
+        <v>WhatsApp</v>
       </c>
       <c r="G2" t="str">
-        <v>wefghj,mnb</v>
+        <v>Received a very long message saying drinking hot garlic water every morning kills the virus before it reaches the lungs. It attributes the claim to a 'Stanford Medical Researcher'.</v>
       </c>
       <c r="H2" t="str">
-        <v>18.654475</v>
+        <v>18.5204</v>
       </c>
       <c r="I2" t="str">
-        <v>73.744029</v>
+        <v>73.8567</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>Pune, Maharashtra</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1713510000000</v>
+        <v>1713513600000</v>
       </c>
       <c r="B3" t="str">
         <v>18/4/2026</v>
       </c>
       <c r="C3" t="str">
-        <v>Verified Fake</v>
+        <v>Pending</v>
       </c>
       <c r="D3" t="str">
-        <v>Rahul_Sharma</v>
+        <v>Priya_Patil</v>
       </c>
       <c r="E3" t="str">
-        <v>WhatsApp forward claiming garlic cures the new virus</v>
+        <v>Video of politician making controversial statements</v>
       </c>
       <c r="F3" t="str">
-        <v>WhatsApp</v>
+        <v>Twitter</v>
       </c>
       <c r="G3" t="str">
-        <v>Received a very long message saying drinking hot garlic water every morning kills the virus before it reaches the lungs. It attributes the claim to a 'Stanford Medical Researcher'.</v>
+        <v>A viral video shows a local politician seemingly admitting to taking bribes. The audio sounds slightly robotic and the mouth movements don't perfectly match the words.</v>
       </c>
       <c r="H3" t="str">
-        <v>18.5204</v>
+        <v>19.0760</v>
       </c>
       <c r="I3" t="str">
-        <v>73.8567</v>
+        <v>72.8777</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>https://twitter.com/example/status/123</v>
       </c>
       <c r="K3" t="str">
-        <v>Pune, Maharashtra</v>
+        <v>Mumbai, Maharashtra</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1713513600000</v>
+        <v>1713520000000</v>
       </c>
       <c r="B4" t="str">
-        <v>18/4/2026</v>
+        <v>19/4/2026</v>
       </c>
       <c r="C4" t="str">
-        <v>Pending</v>
+        <v>Verified True</v>
       </c>
       <c r="D4" t="str">
-        <v>Priya_Patil</v>
+        <v>Admin_User</v>
       </c>
       <c r="E4" t="str">
-        <v>Video of politician making controversial statements</v>
+        <v>Image of severe flooding in city center</v>
       </c>
       <c r="F4" t="str">
-        <v>Twitter</v>
+        <v>Facebook</v>
       </c>
       <c r="G4" t="str">
-        <v>A viral video shows a local politician seemingly admitting to taking bribes. The audio sounds slightly robotic and the mouth movements don't perfectly match the words.</v>
+        <v>Photo going viral showing major roads completely underwater. I live nearby and it rained heavily, but I don't think it's this bad.</v>
       </c>
       <c r="H4" t="str">
-        <v>19.0760</v>
+        <v/>
       </c>
       <c r="I4" t="str">
-        <v>72.8777</v>
+        <v/>
       </c>
       <c r="J4" t="str">
-        <v>https://twitter.com/example/status/123</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Mumbai, Maharashtra</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>1713520000000</v>
+        <v>1713525000000</v>
       </c>
       <c r="B5" t="str">
         <v>19/4/2026</v>
       </c>
       <c r="C5" t="str">
-        <v>Verified True</v>
+        <v>Verified Fake</v>
       </c>
       <c r="D5" t="str">
-        <v>Admin_User</v>
+        <v>Student_Reporter</v>
       </c>
       <c r="E5" t="str">
-        <v>Image of severe flooding in city center</v>
+        <v>Free laptops for all college students via Govt scheme</v>
       </c>
       <c r="F5" t="str">
-        <v>Facebook</v>
+        <v>Telegram</v>
       </c>
       <c r="G5" t="str">
-        <v>Photo going viral showing major roads completely underwater. I live nearby and it rained heavily, but I don't think it's this bad.</v>
+        <v>A link is being shared in groups asking students to enter their Aadhaar and bank details to claim a free laptop from a supposed new government scheme. The URL looks suspicious (gov-scheme-offer.biz).</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>28.6139</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>77.2090</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>http://gov-scheme-offer.biz/laptops</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Delhi</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>1713525000000</v>
+        <v>1713530000000</v>
       </c>
       <c r="B6" t="str">
-        <v>19/4/2026</v>
+        <v>20/4/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Verified Fake</v>
       </c>
       <c r="D6" t="str">
-        <v>Baswaraj_Mundkar</v>
+        <v>DelhiVerifier</v>
       </c>
       <c r="E6" t="str">
-        <v>Free laptops for all college students via Govt scheme</v>
+        <v>Misleading pollution statistics shared during Delhi peak hours</v>
       </c>
       <c r="F6" t="str">
-        <v>Telegram</v>
+        <v>Twitter</v>
       </c>
       <c r="G6" t="str">
-        <v>A link is being shared in groups asking students to enter their Aadhaar and bank details to claim a free laptop from a supposed new government scheme. The URL looks suspicious (gov-scheme-offer.biz).</v>
+        <v>A tweet sharing an AI-generated image of black smog in Connaught Place, falsely claiming AQI reached 999. In reality, it was slightly hazy.</v>
       </c>
       <c r="H6" t="str">
-        <v>28.6139</v>
+        <v>28.6315</v>
       </c>
       <c r="I6" t="str">
-        <v>77.2090</v>
+        <v>77.2167</v>
       </c>
       <c r="J6" t="str">
-        <v>http://gov-scheme-offer.biz/laptops</v>
+        <v>https://twitter.com/example/status/888</v>
       </c>
       <c r="K6" t="str">
-        <v>Delhi</v>
+        <v>New Delhi</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>1713530000000</v>
+        <v>1713535000000</v>
       </c>
       <c r="B7" t="str">
         <v>20/4/2026</v>
       </c>
       <c r="C7" t="str">
-        <v>Verified Fake</v>
+        <v>Pending</v>
       </c>
       <c r="D7" t="str">
-        <v>DelhiVerifier</v>
+        <v>Ramesh_K</v>
       </c>
       <c r="E7" t="str">
-        <v>Misleading pollution statistics shared during Delhi peak hours</v>
+        <v>Scam link promising free water distribution in Bangalore</v>
       </c>
       <c r="F7" t="str">
-        <v>Twitter</v>
+        <v>Facebook</v>
       </c>
       <c r="G7" t="str">
-        <v>A tweet sharing an AI-generated image of black smog in Connaught Place, falsely claiming AQI reached 999. In reality, it was slightly hazy.</v>
+        <v>During the water scarcity, a fake Facebook page impersonating BBMP is asking for Rs. 500 registration fee to get a free tanker.</v>
       </c>
       <c r="H7" t="str">
-        <v>28.6315</v>
+        <v>12.9716</v>
       </c>
       <c r="I7" t="str">
-        <v>77.2167</v>
+        <v>77.5946</v>
       </c>
       <c r="J7" t="str">
-        <v>https://twitter.com/example/status/888</v>
+        <v>http://bbmp-water-free.org</v>
       </c>
       <c r="K7" t="str">
-        <v>New Delhi</v>
+        <v>Bangalore</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>1713535000000</v>
+        <v>1713540000000</v>
       </c>
       <c r="B8" t="str">
-        <v>20/4/2026</v>
+        <v>21/4/2026</v>
       </c>
       <c r="C8" t="str">
-        <v>Pending</v>
+        <v>Verified Fake</v>
       </c>
       <c r="D8" t="str">
-        <v>Ramesh_K</v>
+        <v>Student_Council</v>
       </c>
       <c r="E8" t="str">
-        <v>Scam link promising free water distribution in Bangalore</v>
+        <v>Rumors about PCCOER college closure due to festival</v>
       </c>
       <c r="F8" t="str">
-        <v>Facebook</v>
+        <v>WhatsApp</v>
       </c>
       <c r="G8" t="str">
-        <v>During the water scarcity, a fake Facebook page impersonating BBMP is asking for Rs. 500 registration fee to get a free tanker.</v>
+        <v>A fake notice with the PCCOER letterhead is circulating claiming a 10-day holiday. The college administration confirmed it's forged.</v>
       </c>
       <c r="H8" t="str">
-        <v>12.9716</v>
+        <v>18.6500</v>
       </c>
       <c r="I8" t="str">
-        <v>77.5946</v>
+        <v>73.7500</v>
       </c>
       <c r="J8" t="str">
-        <v>http://bbmp-water-free.org</v>
+        <v/>
       </c>
       <c r="K8" t="str">
-        <v>Bangalore</v>
+        <v>Pune, Ravet</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>1713540000000</v>
+        <v>1713545000000</v>
       </c>
       <c r="B9" t="str">
         <v>21/4/2026</v>
       </c>
       <c r="C9" t="str">
-        <v>Verified Fake</v>
+        <v>Verified True</v>
       </c>
       <c r="D9" t="str">
-        <v>Student_Council</v>
+        <v>Goa_Environment_Group</v>
       </c>
       <c r="E9" t="str">
-        <v>Rumors about PCCOER college closure due to festival</v>
+        <v>Old beach cleaning photos shared as current Goa cleanup</v>
       </c>
       <c r="F9" t="str">
-        <v>WhatsApp</v>
+        <v>Instagram</v>
       </c>
       <c r="G9" t="str">
-        <v>A fake notice with the PCCOER letterhead is circulating claiming a 10-day holiday. The college administration confirmed it's forged.</v>
+        <v>Images from a 2018 cleanup are being shared to promote a fake fundraising campaign.</v>
       </c>
       <c r="H9" t="str">
-        <v>18.6500</v>
+        <v>15.2993</v>
       </c>
       <c r="I9" t="str">
-        <v>73.7500</v>
+        <v>74.1240</v>
       </c>
       <c r="J9" t="str">
         <v/>
       </c>
       <c r="K9" t="str">
-        <v>Pune, Ravet</v>
+        <v>Goa</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>1713545000000</v>
+        <v>1713550000000</v>
       </c>
       <c r="B10" t="str">
-        <v>21/4/2026</v>
+        <v>22/4/2026</v>
       </c>
       <c r="C10" t="str">
-        <v>Verified True</v>
+        <v>Verified Fake</v>
       </c>
       <c r="D10" t="str">
-        <v>Goa_Environment_Group</v>
+        <v>Banker_Anon</v>
       </c>
       <c r="E10" t="str">
-        <v>Old beach cleaning photos shared as current Goa cleanup</v>
+        <v>Viral alert about fake Rs 500 notes in Hyderabad</v>
       </c>
       <c r="F10" t="str">
-        <v>Instagram</v>
+        <v>Telegram</v>
       </c>
       <c r="G10" t="str">
-        <v>Images from a 2018 cleanup are being shared to promote a fake fundraising campaign.</v>
+        <v>A massive chain message telling people to reject notes ending with the series '123'. RBI confirmed this is a rumor.</v>
       </c>
       <c r="H10" t="str">
-        <v>15.2993</v>
+        <v>17.3850</v>
       </c>
       <c r="I10" t="str">
-        <v>74.1240</v>
+        <v>78.4867</v>
       </c>
       <c r="J10" t="str">
         <v/>
       </c>
       <c r="K10" t="str">
-        <v>Goa</v>
+        <v>Hyderabad</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>1713550000000</v>
+        <v>1713555000000</v>
       </c>
       <c r="B11" t="str">
         <v>22/4/2026</v>
       </c>
       <c r="C11" t="str">
-        <v>Verified Fake</v>
+        <v>Verified True</v>
       </c>
       <c r="D11" t="str">
-        <v>Banker_Anon</v>
+        <v>Citizen_O</v>
       </c>
       <c r="E11" t="str">
-        <v>Viral alert about fake Rs 500 notes in Hyderabad</v>
+        <v>Earthquake tremors in Chennai</v>
       </c>
       <c r="F11" t="str">
-        <v>Telegram</v>
+        <v>Twitter</v>
       </c>
       <c r="G11" t="str">
-        <v>A massive chain message telling people to reject notes ending with the series '123'. RBI confirmed this is a rumor.</v>
+        <v>Many users are claiming they felt light tremors in IT corridor.</v>
       </c>
       <c r="H11" t="str">
-        <v>17.3850</v>
+        <v>13.0827</v>
       </c>
       <c r="I11" t="str">
-        <v>78.4867</v>
+        <v>80.2707</v>
       </c>
       <c r="J11" t="str">
         <v/>
       </c>
       <c r="K11" t="str">
-        <v>Hyderabad</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>1713555000000</v>
-      </c>
-      <c r="B12" t="str">
-        <v>22/4/2026</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Verified True</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Citizen_O</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Earthquake tremors in Chennai</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Twitter</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Many users are claiming they felt light tremors in IT corridor.</v>
-      </c>
-      <c r="H12" t="str">
-        <v>13.0827</v>
-      </c>
-      <c r="I12" t="str">
-        <v>80.2707</v>
-      </c>
-      <c r="J12" t="str">
-        <v/>
-      </c>
-      <c r="K12" t="str">
         <v>Chennai</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sanitize repository for public release
</commit_message>
<xml_diff>
--- a/reports.xlsx
+++ b/reports.xlsx
@@ -397,393 +397,429 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>ID</v>
       </c>
       <c r="B1" t="str">
+        <v>Headline</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Image</v>
+      </c>
+      <c r="F1" t="str">
+        <v>URL</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="I1" t="str">
         <v>Date</v>
       </c>
-      <c r="C1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="D1" t="str">
+      <c r="J1" t="str">
         <v>Name</v>
       </c>
-      <c r="E1" t="str">
-        <v>Headline</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Platform</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="H1" t="str">
+      <c r="K1" t="str">
         <v>Lat</v>
       </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>Lng</v>
-      </c>
-      <c r="J1" t="str">
-        <v>URL</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Location</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>1713510000000</v>
+        <v>1713510001001</v>
       </c>
       <c r="B2" t="str">
-        <v>18/4/2026</v>
+        <v>Viral claim that boiling garlic water cures seasonal influenza</v>
       </c>
       <c r="C2" t="str">
+        <v>WhatsApp</v>
+      </c>
+      <c r="D2" t="str">
+        <v>A circulating forward claims drinking boiled garlic water every morning immediately kills respiratory virus particles. Fact-checkers have debunked this as unproven folk medicine.</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v>https://example.com/factcheck/garlic-hoax</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Pune, Maharashtra</v>
+      </c>
+      <c r="H2" t="str">
         <v>Verified Fake</v>
       </c>
-      <c r="D2" t="str">
-        <v>Rahul_Sharma</v>
-      </c>
-      <c r="E2" t="str">
-        <v>WhatsApp forward claiming garlic cures the new virus</v>
-      </c>
-      <c r="F2" t="str">
-        <v>WhatsApp</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Received a very long message saying drinking hot garlic water every morning kills the virus before it reaches the lungs. It attributes the claim to a 'Stanford Medical Researcher'.</v>
-      </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
+        <v>18/04/2026</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Citizen_Verifier</v>
+      </c>
+      <c r="K2" t="str">
         <v>18.5204</v>
       </c>
-      <c r="I2" t="str">
+      <c r="L2" t="str">
         <v>73.8567</v>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v>Pune, Maharashtra</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1713513600000</v>
+        <v>1713510002002</v>
       </c>
       <c r="B3" t="str">
-        <v>18/4/2026</v>
+        <v>Manipulated video snippet of municipal official regarding tax rates</v>
       </c>
       <c r="C3" t="str">
+        <v>Twitter</v>
+      </c>
+      <c r="D3" t="str">
+        <v>A short 10-second video cropped from a 45-minute press conference makes it appear that property taxes will double. The original press conference showed the opposite context.</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>https://example.com/video-snippet</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Mumbai, Maharashtra</v>
+      </c>
+      <c r="H3" t="str">
         <v>Pending</v>
       </c>
-      <c r="D3" t="str">
-        <v>Priya_Patil</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Video of politician making controversial statements</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Twitter</v>
-      </c>
-      <c r="G3" t="str">
-        <v>A viral video shows a local politician seemingly admitting to taking bribes. The audio sounds slightly robotic and the mouth movements don't perfectly match the words.</v>
-      </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
+        <v>18/04/2026</v>
+      </c>
+      <c r="J3" t="str">
+        <v>MediaWatch_Demo</v>
+      </c>
+      <c r="K3" t="str">
         <v>19.0760</v>
       </c>
-      <c r="I3" t="str">
+      <c r="L3" t="str">
         <v>72.8777</v>
-      </c>
-      <c r="J3" t="str">
-        <v>https://twitter.com/example/status/123</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Mumbai, Maharashtra</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1713520000000</v>
+        <v>1713510003003</v>
       </c>
       <c r="B4" t="str">
-        <v>19/4/2026</v>
+        <v>Met Department issues orange alert for heavy coastal rainfall</v>
       </c>
       <c r="C4" t="str">
+        <v>Twitter</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Official advisory issued by the regional meteorological center warning of heavy winds and high tides over the weekend.</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>https://example.gov.in/weather-alert</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Chennai, Tamil Nadu</v>
+      </c>
+      <c r="H4" t="str">
         <v>Verified True</v>
       </c>
-      <c r="D4" t="str">
-        <v>Admin_User</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Image of severe flooding in city center</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Facebook</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Photo going viral showing major roads completely underwater. I live nearby and it rained heavily, but I don't think it's this bad.</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
       <c r="I4" t="str">
-        <v/>
+        <v>19/04/2026</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>Civic_Reporter</v>
+      </c>
+      <c r="K4" t="str">
+        <v>13.0827</v>
+      </c>
+      <c r="L4" t="str">
+        <v>80.2707</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>1713525000000</v>
+        <v>1713510004004</v>
       </c>
       <c r="B5" t="str">
-        <v>19/4/2026</v>
+        <v>Phishing link offering free laptop vouchers under fictitious ministry scheme</v>
       </c>
       <c r="C5" t="str">
+        <v>Telegram</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Suspicious website link promising students high-end laptops after submitting national identity numbers and paying a processing fee. Confirmed phishing portal.</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>http://example-scheme-portal.net</v>
+      </c>
+      <c r="G5" t="str">
+        <v>New Delhi</v>
+      </c>
+      <c r="H5" t="str">
         <v>Verified Fake</v>
       </c>
-      <c r="D5" t="str">
-        <v>Student_Reporter</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Free laptops for all college students via Govt scheme</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Telegram</v>
-      </c>
-      <c r="G5" t="str">
-        <v>A link is being shared in groups asking students to enter their Aadhaar and bank details to claim a free laptop from a supposed new government scheme. The URL looks suspicious (gov-scheme-offer.biz).</v>
-      </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
+        <v>19/04/2026</v>
+      </c>
+      <c r="J5" t="str">
+        <v>FactCheck_Volunteer</v>
+      </c>
+      <c r="K5" t="str">
         <v>28.6139</v>
       </c>
-      <c r="I5" t="str">
+      <c r="L5" t="str">
         <v>77.2090</v>
-      </c>
-      <c r="J5" t="str">
-        <v>http://gov-scheme-offer.biz/laptops</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Delhi</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>1713530000000</v>
+        <v>1713510005005</v>
       </c>
       <c r="B6" t="str">
-        <v>20/4/2026</v>
+        <v>Fabricated university holiday circular shared during examination week</v>
       </c>
       <c r="C6" t="str">
+        <v>WhatsApp</v>
+      </c>
+      <c r="D6" t="str">
+        <v>A forged university letterhead claiming exams have been postponed due to a sudden declared holiday. University authorities issued a clarification stating exams proceed as scheduled.</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>https://example-university.edu/notice</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Pune, Maharashtra</v>
+      </c>
+      <c r="H6" t="str">
         <v>Verified Fake</v>
       </c>
-      <c r="D6" t="str">
-        <v>DelhiVerifier</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Misleading pollution statistics shared during Delhi peak hours</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Twitter</v>
-      </c>
-      <c r="G6" t="str">
-        <v>A tweet sharing an AI-generated image of black smog in Connaught Place, falsely claiming AQI reached 999. In reality, it was slightly hazy.</v>
-      </c>
-      <c r="H6" t="str">
-        <v>28.6315</v>
-      </c>
       <c r="I6" t="str">
-        <v>77.2167</v>
+        <v>20/04/2026</v>
       </c>
       <c r="J6" t="str">
-        <v>https://twitter.com/example/status/888</v>
+        <v>Student_Observer</v>
       </c>
       <c r="K6" t="str">
-        <v>New Delhi</v>
+        <v>18.6500</v>
+      </c>
+      <c r="L6" t="str">
+        <v>73.7500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>1713535000000</v>
+        <v>1713510006006</v>
       </c>
       <c r="B7" t="str">
-        <v>20/4/2026</v>
+        <v>Fraudulent tanker booking page asking advance fees during water repair</v>
       </c>
       <c r="C7" t="str">
+        <v>Facebook</v>
+      </c>
+      <c r="D7" t="str">
+        <v>A counterfeit social media page claiming to provide immediate private water tankers for a registration fee. Community alerts issued to book only via official helpline.</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>http://water-supply-sample.org</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Bengaluru, Karnataka</v>
+      </c>
+      <c r="H7" t="str">
         <v>Pending</v>
       </c>
-      <c r="D7" t="str">
-        <v>Ramesh_K</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Scam link promising free water distribution in Bangalore</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Facebook</v>
-      </c>
-      <c r="G7" t="str">
-        <v>During the water scarcity, a fake Facebook page impersonating BBMP is asking for Rs. 500 registration fee to get a free tanker.</v>
-      </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
+        <v>20/04/2026</v>
+      </c>
+      <c r="J7" t="str">
+        <v>DigitalLiteracy_User</v>
+      </c>
+      <c r="K7" t="str">
         <v>12.9716</v>
       </c>
-      <c r="I7" t="str">
+      <c r="L7" t="str">
         <v>77.5946</v>
-      </c>
-      <c r="J7" t="str">
-        <v>http://bbmp-water-free.org</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Bangalore</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>1713540000000</v>
+        <v>1713510007007</v>
       </c>
       <c r="B8" t="str">
-        <v>21/4/2026</v>
+        <v>Community beach clean-up drive organized by registered environmental NGO</v>
       </c>
       <c r="C8" t="str">
-        <v>Verified Fake</v>
+        <v>Instagram</v>
       </c>
       <c r="D8" t="str">
-        <v>Student_Council</v>
+        <v>Photos of volunteers clearing marine debris along Miramar coast verified as an authentic scheduled civic initiative.</v>
       </c>
       <c r="E8" t="str">
-        <v>Rumors about PCCOER college closure due to festival</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>WhatsApp</v>
+        <v>https://example.org/coastal-drive</v>
       </c>
       <c r="G8" t="str">
-        <v>A fake notice with the PCCOER letterhead is circulating claiming a 10-day holiday. The college administration confirmed it's forged.</v>
+        <v>Panaji, Goa</v>
       </c>
       <c r="H8" t="str">
-        <v>18.6500</v>
+        <v>Verified True</v>
       </c>
       <c r="I8" t="str">
-        <v>73.7500</v>
+        <v>21/04/2026</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>EcoWatch_Reporter</v>
       </c>
       <c r="K8" t="str">
-        <v>Pune, Ravet</v>
+        <v>15.2993</v>
+      </c>
+      <c r="L8" t="str">
+        <v>74.1240</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>1713545000000</v>
+        <v>1713510008008</v>
       </c>
       <c r="B9" t="str">
-        <v>21/4/2026</v>
+        <v>Hoax audio message alleging demonetization of specific currency denominations</v>
       </c>
       <c r="C9" t="str">
-        <v>Verified True</v>
+        <v>WhatsApp</v>
       </c>
       <c r="D9" t="str">
-        <v>Goa_Environment_Group</v>
+        <v>Viral audio claim urging citizens to exchange specific currency notes within 48 hours. Central bank confirmed currency remains valid and legal tender.</v>
       </c>
       <c r="E9" t="str">
-        <v>Old beach cleaning photos shared as current Goa cleanup</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v>Instagram</v>
+        <v>https://example-banking.org/statement</v>
       </c>
       <c r="G9" t="str">
-        <v>Images from a 2018 cleanup are being shared to promote a fake fundraising campaign.</v>
+        <v>Hyderabad, Telangana</v>
       </c>
       <c r="H9" t="str">
-        <v>15.2993</v>
+        <v>Verified Fake</v>
       </c>
       <c r="I9" t="str">
-        <v>74.1240</v>
+        <v>21/04/2026</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>Community_Verifier</v>
       </c>
       <c r="K9" t="str">
-        <v>Goa</v>
+        <v>17.3850</v>
+      </c>
+      <c r="L9" t="str">
+        <v>78.4867</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>1713550000000</v>
+        <v>1713510009009</v>
       </c>
       <c r="B10" t="str">
-        <v>22/4/2026</v>
+        <v>Digitally altered image claiming air quality index exceeded 999</v>
       </c>
       <c r="C10" t="str">
+        <v>Facebook</v>
+      </c>
+      <c r="D10" t="str">
+        <v>An altered photo with an alarming fake AQI reading circulated online. Official pollution monitors confirmed standard seasonal air quality readings.</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v>https://example.com/aqi-check</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Kolkata, West Bengal</v>
+      </c>
+      <c r="H10" t="str">
         <v>Verified Fake</v>
       </c>
-      <c r="D10" t="str">
-        <v>Banker_Anon</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Viral alert about fake Rs 500 notes in Hyderabad</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Telegram</v>
-      </c>
-      <c r="G10" t="str">
-        <v>A massive chain message telling people to reject notes ending with the series '123'. RBI confirmed this is a rumor.</v>
-      </c>
-      <c r="H10" t="str">
-        <v>17.3850</v>
-      </c>
       <c r="I10" t="str">
-        <v>78.4867</v>
+        <v>22/04/2026</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>NewsMonitor_Demo</v>
       </c>
       <c r="K10" t="str">
-        <v>Hyderabad</v>
+        <v>22.5726</v>
+      </c>
+      <c r="L10" t="str">
+        <v>88.3639</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>1713555000000</v>
+        <v>1713510010010</v>
       </c>
       <c r="B11" t="str">
-        <v>22/4/2026</v>
+        <v>Traffic diversion advisory announced for metro corridor expansion</v>
       </c>
       <c r="C11" t="str">
+        <v>Twitter</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Municipal traffic division notice announcing night-time diversions between Junction 4 and 7 for girder erection work.</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>https://example-traffic.gov.in/advisory</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Ahmedabad, Gujarat</v>
+      </c>
+      <c r="H11" t="str">
         <v>Verified True</v>
       </c>
-      <c r="D11" t="str">
-        <v>Citizen_O</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Earthquake tremors in Chennai</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Twitter</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Many users are claiming they felt light tremors in IT corridor.</v>
-      </c>
-      <c r="H11" t="str">
-        <v>13.0827</v>
-      </c>
       <c r="I11" t="str">
-        <v>80.2707</v>
+        <v>22/04/2026</v>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>SafetyWatch_User</v>
       </c>
       <c r="K11" t="str">
-        <v>Chennai</v>
+        <v>23.0225</v>
+      </c>
+      <c r="L11" t="str">
+        <v>72.5714</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>